<commit_message>
revision6_checks.py: genotype-adjusted lineage models exclude other variants, interaction models, without engineered models; bootstrap seed stability; comparator decomposition for non-blood pairs; S3 Table rows for revision-5/6 analyses
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/supporting_information/S3_Table.xlsx
+++ b/figures/supporting_information/S3_Table.xlsx
@@ -840,7 +840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1002,10 +1002,166 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Growth-pattern adjustment of the 42 blood pairs, with / without the other blood lineage</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>median ratio adjusted/unadjusted 0.56 / 0.84; pairs with q &lt; 0.05 36 / 42 (growth_confound_pairs.csv)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sanger replication by lineage group</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>lymphoid 16/17, other 8/15; non-prioritised reference 294/1182 and 263/1079; failing only the median criterion 18/22</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Bootstrap 95% intervals of selectivity (1,000 resamples, seed 42; per pair in S2 Table)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>entirely below -0.5: 29 pairs (seeds 43-45: 28, 28, 28); below 0: 93</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Median of all other lines, prioritised pairs</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>above -0.5: 40; -1 to -0.5: 41; -1 or below: 13; another eligible lineage below -1: 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Non-blood pairs with other comparison groups (selectivity &lt; -0.5, of 52)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>adherent lines only 42; without suspension lines 45; without blood lines 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CTNNB1 by APC truncating variant</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>median -1.04 (n = 78) vs -0.13 (n = 1023); lineage-adjusted difference -0.54, p = 5.7e-26; within lineage -1.34 (n = 49) vs -0.52 (n = 9), p = 0.011</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BRAF by BRAF V600 variant</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>median -1.20 (n = 79) vs -0.08 (n = 1067); lineage-adjusted difference -0.97, p = 4.2e-135; within lineage -1.28 (n = 49) vs -0.09 (n = 23), p = 4.8e-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CTNNB1 in bowel by APC/CTNNB1 group</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>APC truncating -1.34 (n = 49); CTNNB1 hotspot -1.76 (n = 4); neither -0.36 (n = 8) vs other lineages -0.13, p = 0.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Lineage coefficient adjusted for genotype, KRAS pancreas</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ratio 0.28 (p = 6.9e-10); interaction model: lineage effect in non-carriers -0.03 (p = 0.91), lineage x genotype -0.43 (p = 0.082)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lineage coefficient adjusted for genotype, CTNNB1 bowel</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ratio 0.50 (p = 3.1e-21); interaction model: lineage effect in non-carriers -0.52 (p = 3.3e-06), lineage x genotype 0.01 (p = 0.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Lineage coefficient adjusted for genotype, BRAF skin</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ratio 0.22 (p = 2.8e-08); interaction model: lineage effect in non-carriers -0.05 (p = 0.29), lineage x genotype -0.31 (p = 4e-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Lineage coefficient adjusted for genotype, BRAF skin without engineered</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ratio 0.27 (p = 2.1e-12); interaction model: lineage effect in non-carriers -0.05 (p = 0.27), lineage x genotype -0.43 (p = 9.9e-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>22Q1 with quantile-matched thresholds (shared lines)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>selectivity -0.41, median -1.05: 31 of 90 pairs meet the rule; selectivity only: 37; original thresholds: 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>22Q1 vs 26Q1 on the same 1,036 models</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>primary pairs meeting the rule: 84 (26Q1 data) vs 23 (22Q1 data)</t>
         </is>

</xml_diff>